<commit_message>
Chore: remove ads from 404 and prune obsolete pages
</commit_message>
<xml_diff>
--- a/seo_inventory_report.xlsx
+++ b/seo_inventory_report.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SEO AdSense 盤點'!$A$1:$K$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SEO AdSense 盤點'!$A$1:$K$154</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -157,8 +157,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SEOInventory" displayName="SEOInventory" ref="A1:K168" headerRowCount="1">
-  <autoFilter ref="A1:K168"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SEOInventory" displayName="SEOInventory" ref="A1:K154" headerRowCount="1">
+  <autoFilter ref="A1:K154"/>
   <tableColumns count="11">
     <tableColumn id="1" name="編號"/>
     <tableColumn id="2" name="頁面分類"/>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K168"/>
+  <dimension ref="A1:K154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -579,7 +579,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 未配置（合規）</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
@@ -3910,17 +3910,17 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>en/contact.html</t>
+          <t>en/index.html</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/contact.html</t>
+          <t>https://gugopro.com/en/index.html</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3930,12 +3930,12 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Contact Us | GugoPro Official</t>
+          <t>GugoPro Official Homepage | AI and Utility Tools</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Contact Us</t>
+          <t>Web AI, data and utility tools for everyday work.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3949,10 +3949,10 @@
         </is>
       </c>
       <c r="J68" s="2" t="n">
-        <v>156</v>
+        <v>108</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69">
@@ -3961,17 +3961,17 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>en/index.html</t>
+          <t>en/tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/index.html</t>
+          <t>https://gugopro.com/en/tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>GugoPro Official Homepage | AI and Utility Tools</t>
+          <t>Redirecting - AI Multilingual Speaking Tutor | GugoPro</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Web AI, data and utility tools for everyday work.</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3996,14 +3996,14 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J69" s="2" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -4012,17 +4012,17 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>en/legal/about.html</t>
+          <t>en/tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/legal/about.html</t>
+          <t>https://gugopro.com/en/tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -4032,12 +4032,12 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>About GugoPro | GugoPro</t>
+          <t>Redirecting - Face-to-Face Travel Voice Translator | GugoPro</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>About GugoPro</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -4047,14 +4047,14 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J70" s="2" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -4063,17 +4063,17 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>en/legal/contact.html</t>
+          <t>en/tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/legal/contact.html</t>
+          <t>https://gugopro.com/en/tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -4083,12 +4083,12 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Contact Us | GugoPro</t>
+          <t>Redirecting - AI Tarot Master | GugoPro</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Contact Us</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -4098,14 +4098,14 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J71" s="2" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -4114,17 +4114,17 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>en/legal/disclaimer.html</t>
+          <t>en/tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/legal/disclaimer.html</t>
+          <t>https://gugopro.com/en/tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -4134,12 +4134,12 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Disclaimer | GugoPro</t>
+          <t>Redirecting - GugoPro AI Ziwei Astrology Master | GugoPro</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Disclaimer</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -4149,14 +4149,14 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>142</v>
+        <v>0</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -4165,17 +4165,17 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>en/legal/privacy.html</t>
+          <t>en/tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/legal/privacy.html</t>
+          <t>https://gugopro.com/en/tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -4185,12 +4185,12 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy | GugoPro</t>
+          <t>Redirecting - YouTube Sequel Tracker | GugoPro</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Privacy Policy</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -4200,14 +4200,14 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J73" s="2" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -4216,17 +4216,17 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>en/legal/terms.html</t>
+          <t>en/tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/legal/terms.html</t>
+          <t>https://gugopro.com/en/tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -4236,12 +4236,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Terms of Service | GugoPro</t>
+          <t>Redirecting - YouTube Study Player | GugoPro</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Terms of Service</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -4251,14 +4251,14 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J74" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -4272,12 +4272,12 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/english-speaking-tutor.html</t>
+          <t>en/tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/english-speaking-tutor.html</t>
+          <t>https://gugopro.com/en/tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - AI Multilingual Speaking Tutor | GugoPro</t>
+          <t>Redirecting - AI Nutritionist | GugoPro</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -4323,12 +4323,12 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/realtime-translator.html</t>
+          <t>en/tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/realtime-translator.html</t>
+          <t>https://gugopro.com/en/tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - Face-to-Face Travel Voice Translator | GugoPro</t>
+          <t>Redirecting - AI Weight Loss Coach | GugoPro</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4369,17 +4369,17 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/tarot-master.html</t>
+          <t>en/tools/pdf/pdf-suite.html</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/tarot-master.html</t>
+          <t>https://gugopro.com/en/tools/pdf/pdf-suite.html</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -4389,7 +4389,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - AI Tarot Master | GugoPro</t>
+          <t>Redirecting - PDF Suite | GugoPro</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -4420,29 +4420,21 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/ziwei-astrology.html</t>
+          <t>googled0dfad57039c64f6.html</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/ziwei-astrology.html</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>Redirecting - GugoPro AI Ziwei Astrology Master | GugoPro</t>
-        </is>
-      </c>
+          <t>https://gugopro.com/googled0dfad57039c64f6.html</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
           <t>❌ 缺失</t>
@@ -4462,7 +4454,7 @@
         <v>0</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -4471,32 +4463,32 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai-media/ai-video-tracker.html</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai-media/ai-video-tracker.html</t>
+          <t>https://gugopro.com/index.html</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - YouTube Sequel Tracker | GugoPro</t>
+          <t>GugoPro 工具箱｜YouTube 雙語字幕學習、AI 翻譯塔羅、TDEE 減脂計算與跨境選品等 10 款免費免安裝工具</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>GugoPro 工具箱</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -4506,14 +4498,14 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0</v>
+        <v>214</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80">
@@ -4522,17 +4514,17 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>en/tools/english/l-player-study.html</t>
+          <t>index_en.html</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/english/l-player-study.html</t>
+          <t>https://gugopro.com/index_en.html</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -4542,12 +4534,12 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - YouTube Study Player | GugoPro</t>
+          <t>GugoPro Hub | 10 Free Browser Tools for YouTube Study, AI Translation &amp; Tarot, TDEE, and Product Research</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>GugoPro Hub</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4557,14 +4549,14 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0</v>
+        <v>396</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81">
@@ -4573,32 +4565,32 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>en/tools/health/tdee-macros-calculator.html</t>
+          <t>index_ja.html</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/health/tdee-macros-calculator.html</t>
+          <t>https://gugopro.com/index_ja.html</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - AI Nutritionist | GugoPro</t>
+          <t>GugoPro ツールボックス｜YouTube 2言語字幕学習、AI 翻訳タロット、TDEE 減脂計算、越境EC商品選定など無料ブラウザツール10選</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>GugoPro ツールボックス</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -4608,14 +4600,14 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0</v>
+        <v>213</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82">
@@ -4624,32 +4616,32 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>en/tools/health/weight-loss-planner.html</t>
+          <t>ja/articles/affective-filter-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/health/weight-loss-planner.html</t>
+          <t>https://gugopro.com/ja/articles/affective-filter-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - AI Weight Loss Coach | GugoPro</t>
+          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド｜GugoPro 言語学習コラム</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -4659,14 +4651,14 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
@@ -4675,32 +4667,32 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>歷史工具</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>en/tools/pdf/pdf-suite.html</t>
+          <t>ja/articles/amazon-ai-product-research-guide.html</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/pdf/pdf-suite.html</t>
+          <t>https://gugopro.com/ja/articles/amazon-ai-product-research-guide.html</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - PDF Suite | GugoPro</t>
+          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス｜GugoPro EC戦略コラム</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -4710,11 +4702,11 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>1</v>
@@ -4726,24 +4718,32 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>googled0dfad57039c64f6.html</t>
+          <t>ja/articles/carb-cycling-and-home-workout-guide.html</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/googled0dfad57039c64f6.html</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr"/>
-      <c r="F84" s="2" t="inlineStr"/>
+          <t>https://gugopro.com/ja/articles/carb-cycling-and-home-workout-guide.html</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意｜GugoPro 運動生理学コラム</t>
+        </is>
+      </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -4753,14 +4753,14 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
@@ -4769,32 +4769,32 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>guides/risk-reward-ratio.html</t>
+          <t>ja/articles/diabetes-and-insulin-resistance-guide.html</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/guides/risk-reward-ratio.html</t>
+          <t>https://gugopro.com/ja/articles/diabetes-and-insulin-resistance-guide.html</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>zh-Hant</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>交易風險報酬比（R:R）｜GugoPro 財經學院</t>
+          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控｜GugoPro 代謝医学コラム</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>交易風險報酬比（R:R）：先理解，再計算，最後管理風險。</t>
+          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -4808,10 +4808,10 @@
         </is>
       </c>
       <c r="J85" s="2" t="n">
-        <v>52</v>
+        <v>164</v>
       </c>
       <c r="K85" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
@@ -4820,32 +4820,32 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>index.html</t>
+          <t>ja/articles/english-intro-break-the-ice.html</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/index.html</t>
+          <t>https://gugopro.com/ja/articles/english-intro-break-the-ice.html</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>zh-TW</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>GugoPro 工具箱｜YouTube 雙語字幕學習、AI 翻譯塔羅、TDEE 減脂計算與跨境選品等 10 款免費免安裝工具</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイング完全ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>GugoPro 工具箱</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -4859,10 +4859,10 @@
         </is>
       </c>
       <c r="J86" s="2" t="n">
-        <v>214</v>
+        <v>170</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
@@ -4871,32 +4871,32 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>index_en.html</t>
+          <t>ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/index_en.html</t>
+          <t>https://gugopro.com/ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>GugoPro Hub | 10 Free Browser Tools for YouTube Study, AI Translation &amp; Tarot, TDEE, and Product Research</t>
+          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル｜GugoPro 肝臓代謝コラム</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>GugoPro Hub</t>
+          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -4910,10 +4910,10 @@
         </is>
       </c>
       <c r="J87" s="2" t="n">
-        <v>396</v>
+        <v>206</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88">
@@ -4922,17 +4922,17 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>index_ja.html</t>
+          <t>ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/index_ja.html</t>
+          <t>https://gugopro.com/ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -4942,12 +4942,12 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>GugoPro ツールボックス｜YouTube 2言語字幕学習、AI 翻訳タロット、TDEE 減脂計算、越境EC商品選定など無料ブラウザツール10選</t>
+          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南｜GugoPro クラウドシステムコラム</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>GugoPro ツールボックス</t>
+          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -4961,10 +4961,10 @@
         </is>
       </c>
       <c r="J88" s="2" t="n">
-        <v>213</v>
+        <v>271</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89">
@@ -4978,12 +4978,12 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/affective-filter-with-ai-tutor.html</t>
+          <t>ja/articles/how-to-master-tarot-guide.html</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/affective-filter-with-ai-tutor.html</t>
+          <t>https://gugopro.com/ja/articles/how-to-master-tarot-guide.html</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -4993,12 +4993,12 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド｜GugoPro 言語学習コラム</t>
+          <t>タロットマスターへの道：78枚の丸暗記を脱し「直観的フロー・リーディング」へ——古典記号論、ナラティブ心理学、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド</t>
+          <t>如何にしてタロットマスターとなるか？ 78枚の意味の丸暗記から「直観的フロー・リーディング」へ：古典記号論・ナラティブ心理学・AI協同による限界的練習完全手引</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="J89" s="2" t="n">
-        <v>221</v>
+        <v>145</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>2</v>
@@ -5029,12 +5029,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/amazon-ai-product-research-guide.html</t>
+          <t>ja/articles/how-to-master-ziwei-guide.html</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/amazon-ai-product-research-guide.html</t>
+          <t>https://gugopro.com/ja/articles/how-to-master-ziwei-guide.html</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -5044,12 +5044,12 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス｜GugoPro EC戦略コラム</t>
+          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス</t>
+          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -5063,10 +5063,10 @@
         </is>
       </c>
       <c r="J90" s="2" t="n">
-        <v>227</v>
+        <v>199</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91">
@@ -5080,12 +5080,12 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/carb-cycling-and-home-workout-guide.html</t>
+          <t>ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/carb-cycling-and-home-workout-guide.html</t>
+          <t>https://gugopro.com/ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -5095,12 +5095,12 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意｜GugoPro 運動生理学コラム</t>
+          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド｜GugoPro 代謝内分泌コラム</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意</t>
+          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="J91" s="2" t="n">
-        <v>204</v>
+        <v>233</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>2</v>
@@ -5131,12 +5131,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/diabetes-and-insulin-resistance-guide.html</t>
+          <t>ja/articles/investment/01-compound-interest-guide.html</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/diabetes-and-insulin-resistance-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/01-compound-interest-guide.html</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -5146,12 +5146,12 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控｜GugoPro 代謝医学コラム</t>
+          <t>複利効果と時間価値：バランスシートから最初のファイナンシャルシステムを構築するには？ | GugoPro Academy</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控</t>
+          <t>複利効果と時間価値：バランスシートから最初のファイナンシャルシステムを構築するには？</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -5165,10 +5165,10 @@
         </is>
       </c>
       <c r="J92" s="2" t="n">
-        <v>164</v>
+        <v>43</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -5182,12 +5182,12 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/english-intro-break-the-ice.html</t>
+          <t>ja/articles/investment/02-etf-investing-bible.html</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/english-intro-break-the-ice.html</t>
+          <t>https://gugopro.com/ja/articles/investment/02-etf-investing-bible.html</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -5197,12 +5197,12 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイング完全ガイド｜GugoPro 言語科学コラム</t>
+          <t>インデックス投資バイブル：台湾 0050/006208 vs 米国 VTI/VOO/QQQ 完全解析 | GugoPro Academy</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
+          <t>インデックス投資バイブル：台湾 0050/006208 vs 米国 VTI/VOO/QQQ 完全解析</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -5216,10 +5216,10 @@
         </is>
       </c>
       <c r="J93" s="2" t="n">
-        <v>170</v>
+        <v>63</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -5233,12 +5233,12 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
+          <t>ja/articles/investment/03-asset-allocation-rebalancing.html</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/03-asset-allocation-rebalancing.html</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -5248,12 +5248,12 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル｜GugoPro 肝臓代謝コラム</t>
+          <t>資産配分と動的リバランス：目標ウェイトから取引摩擦まで｜GugoPro Academy</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル</t>
+          <t>資産配分と動的リバランス： 目標ウェイトを実行可能な意思決定ルールにする。</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -5267,10 +5267,10 @@
         </is>
       </c>
       <c r="J94" s="2" t="n">
-        <v>206</v>
+        <v>88</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -5284,12 +5284,12 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
+          <t>ja/articles/investment/04-brokerage-comparison.html</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/04-brokerage-comparison.html</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -5299,12 +5299,12 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南｜GugoPro クラウドシステムコラム</t>
+          <t>米国ブローカー口座開設完全ガイド：台湾の複委託 vs 海外ブローカー | GugoPro Academy</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南</t>
+          <t>米国ブローカー口座開設完全ガイド：台湾の複委託 vs 海外ブローカー（Firstrade、IB、Schwab）比較</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -5318,10 +5318,10 @@
         </is>
       </c>
       <c r="J95" s="2" t="n">
-        <v>271</v>
+        <v>63</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/how-to-master-tarot-guide.html</t>
+          <t>ja/articles/investment/05-fundamental-valuation-metrics.html</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/how-to-master-tarot-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/05-fundamental-valuation-metrics.html</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -5350,12 +5350,12 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>タロットマスターへの道：78枚の丸暗記を脱し「直観的フロー・リーディング」へ——古典記号論、ナラティブ心理学、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
+          <t>ファンダメンタル評価指標：P/E、P/B、ROE | GugoPro Academy</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>如何にしてタロットマスターとなるか？ 78枚の意味の丸暗記から「直観的フロー・リーディング」へ：古典記号論・ナラティブ心理学・AI協同による限界的練習完全手引</t>
+          <t>ファンダメンタル評価指標：P/E（株価収益率）、P/B（株価純資産倍率）、ROEの正しい読み方</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -5369,10 +5369,10 @@
         </is>
       </c>
       <c r="J96" s="2" t="n">
-        <v>145</v>
+        <v>61</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -5386,12 +5386,12 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/how-to-master-ziwei-guide.html</t>
+          <t>ja/articles/investment/06-sharpe-mdd-risk-control.html</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/how-to-master-ziwei-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/06-sharpe-mdd-risk-control.html</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -5401,12 +5401,12 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
+          <t>リスクリターンと最大ドローダウン分析：Sharpe、Sortino、Calmar 実装ガイド｜GugoPro Academy</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド</t>
+          <t>リスクリターンと最大ドローダウンの分析</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -5420,10 +5420,10 @@
         </is>
       </c>
       <c r="J97" s="2" t="n">
-        <v>199</v>
+        <v>108</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -5437,12 +5437,12 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
+          <t>ja/articles/investment/07-fire-4-percent-rule.html</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/07-fire-4-percent-rule.html</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -5452,12 +5452,12 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド｜GugoPro 代謝内分泌コラム</t>
+          <t>【退職金プラン】FIRE ムーブメントと 4% ルールとは？引き出し率と退職資金の不足額の計算方法 | GugoPro Academy</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド</t>
+          <t>【退職金プラン】FIRE ムーブメントと 4% ルールとは？引き出し率と退職資金の不足額の計算方法</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -5471,10 +5471,10 @@
         </is>
       </c>
       <c r="J98" s="2" t="n">
-        <v>233</v>
+        <v>85</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -5488,12 +5488,12 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/01-compound-interest-guide.html</t>
+          <t>ja/articles/investment/08-overseas-tax-guide.html</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/01-compound-interest-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/08-overseas-tax-guide.html</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -5503,12 +5503,12 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>複利効果と時間価値：バランスシートから最初のファイナンシャルシステムを構築するには？ | GugoPro Academy</t>
+          <t>【節税と確定申告】米国株投資はどう申告するか？海外所得 750 萬 の免税枠と 30% 配当源泉徴収の実務 | GugoPro Academy</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>複利効果と時間価値：バランスシートから最初のファイナンシャルシステムを構築するには？</t>
+          <t>【節税と確定申告】米国株投資はどう申告するか？海外所得 750 萬 の免税枠と 30% 配当源泉徴収の実務</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -5522,10 +5522,10 @@
         </is>
       </c>
       <c r="J99" s="2" t="n">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -5539,12 +5539,12 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/02-etf-investing-bible.html</t>
+          <t>ja/articles/investment/09-high-dividend-etf-trap.html</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/02-etf-investing-bible.html</t>
+          <t>https://gugopro.com/ja/articles/investment/09-high-dividend-etf-trap.html</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -5554,12 +5554,12 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>インデックス投資バイブル：台湾 0050/006208 vs 米国 VTI/VOO/QQQ 完全解析 | GugoPro Academy</t>
+          <t>【高配当 ETF 評価】台湾上場 ETF 00878/00919/00929 vs 米国 ETF SCHD：高配当利回りの罠を解くと総リターンの真実が見える | GugoPro Academy</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>インデックス投資バイブル：台湾 0050/006208 vs 米国 VTI/VOO/QQQ 完全解析</t>
+          <t>【高配当 ETF 評価】台湾上場 ETF 00878/00919/00929 vs 米国 ETF SCHD：高配当利回りの罠を解くと総リターンの真実が見える</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -5573,7 +5573,7 @@
         </is>
       </c>
       <c r="J100" s="2" t="n">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5590,12 +5590,12 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/03-asset-allocation-rebalancing.html</t>
+          <t>ja/articles/investment/10-bond-investing-guide.html</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/03-asset-allocation-rebalancing.html</t>
+          <t>https://gugopro.com/ja/articles/investment/10-bond-investing-guide.html</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -5605,12 +5605,12 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>資産配分と動的リバランス：目標ウェイトから取引摩擦まで｜GugoPro Academy</t>
+          <t>【債券投資ガイド】米国債 (TLT/IEF) vs 投資適格社債 (LQD)：利下げサイクルにおける資産配分戦略 | GugoPro Academy</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>資産配分と動的リバランス： 目標ウェイトを実行可能な意思決定ルールにする。</t>
+          <t>【債券投資ガイド】米国債 (TLT/IEF) vs 投資適格社債 (LQD)：利下げサイクルにおける資産配分戦略</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="J101" s="2" t="n">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5641,12 +5641,12 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/04-brokerage-comparison.html</t>
+          <t>ja/articles/investment/11-brokerage-deep-review.html</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/04-brokerage-comparison.html</t>
+          <t>https://gugopro.com/ja/articles/investment/11-brokerage-deep-review.html</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -5656,12 +5656,12 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>米国ブローカー口座開設完全ガイド：台湾の複委託 vs 海外ブローカー | GugoPro Academy</t>
+          <t>【海外証券会社評価大全】IB（盈透／Interactive Brokers）、Firstrade、Charles Schwab（嘉信理財）─ 長所・短所、安全性と隠れたコスト比較 | GugoPro Academy</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>米国ブローカー口座開設完全ガイド：台湾の複委託 vs 海外ブローカー（Firstrade、IB、Schwab）比較</t>
+          <t>【海外証券会社評価大全】IB（盈透／Interactive Brokers）、Firstrade、Charles Schwab（嘉信理財）─ 長所・短所、安全性と隠れたコスト比較</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -5675,7 +5675,7 @@
         </is>
       </c>
       <c r="J102" s="2" t="n">
-        <v>63</v>
+        <v>111</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5692,12 +5692,12 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/05-fundamental-valuation-metrics.html</t>
+          <t>ja/articles/investment/12-inflation-hedging-reits-gold.html</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/05-fundamental-valuation-metrics.html</t>
+          <t>https://gugopro.com/ja/articles/investment/12-inflation-hedging-reits-gold.html</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -5707,12 +5707,12 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>ファンダメンタル評価指標：P/E、P/B、ROE | GugoPro Academy</t>
+          <t>【ヘッジ資産】金（GLD）と不動産投資信託（REITs）はインフレ対策として資産配分にどう組み込むか？ | GugoPro Academy</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>ファンダメンタル評価指標：P/E（株価収益率）、P/B（株価純資産倍率）、ROEの正しい読み方</t>
+          <t>【ヘッジ資産】金（GLD）と不動産投資信託（REITs）はインフレ対策として資産配分にどう組み込むか？</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
@@ -5726,7 +5726,7 @@
         </is>
       </c>
       <c r="J103" s="2" t="n">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5743,12 +5743,12 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/06-sharpe-mdd-risk-control.html</t>
+          <t>ja/articles/investment/13-technical-indicators-truth.html</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/06-sharpe-mdd-risk-control.html</t>
+          <t>https://gugopro.com/ja/articles/investment/13-technical-indicators-truth.html</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -5758,12 +5758,12 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>リスクリターンと最大ドローダウン分析：Sharpe、Sortino、Calmar 実装ガイド｜GugoPro Academy</t>
+          <t>【テクニカル分析の真実】移動平均線 (MA)、RSI、MACD は本当に役立つのか？クオンツトレーダーが見るテクニカル指標の有効場面と盲点 | GugoPro Academy</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>リスクリターンと最大ドローダウンの分析</t>
+          <t>【テクニカル分析の真実】移動平均線 (MA)、RSI、MACD は本当に役立つのか？クオンツトレーダーが見るテクニカル指標の有効場面と盲点</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -5777,7 +5777,7 @@
         </is>
       </c>
       <c r="J104" s="2" t="n">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5794,12 +5794,12 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/07-fire-4-percent-rule.html</t>
+          <t>ja/articles/investment/14-backtesting-overfitting-guide.html</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/07-fire-4-percent-rule.html</t>
+          <t>https://gugopro.com/ja/articles/investment/14-backtesting-overfitting-guide.html</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -5809,12 +5809,12 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>【退職金プラン】FIRE ムーブメントと 4% ルールとは？引き出し率と退職資金の不足額の計算方法 | GugoPro Academy</t>
+          <t>【システムトレード】バックテスト (Backtesting/回測) とは？過学習 (Overfitting/過度擬合) と歴史的罠を避ける方法 | GugoPro Academy</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>【退職金プラン】FIRE ムーブメントと 4% ルールとは？引き出し率と退職資金の不足額の計算方法</t>
+          <t>【システムトレード】バックテスト (Backtesting/回測) とは？過学習 (Overfitting/過度擬合) と歴史的罠を避ける方法</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -5828,7 +5828,7 @@
         </is>
       </c>
       <c r="J105" s="2" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -5845,12 +5845,12 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/08-overseas-tax-guide.html</t>
+          <t>ja/articles/investment/15-quant-research-workflow.html</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/08-overseas-tax-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/15-quant-research-workflow.html</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -5860,12 +5860,12 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>【節税と確定申告】米国株投資はどう申告するか？海外所得 750 萬 の免税枠と 30% 配当源泉徴収の実務 | GugoPro Academy</t>
+          <t>量的研究ワークフロー：5MAオフセット、ボラティリティのZ‑Score、アウト‑オブ‑サンプルバックテスト｜GugoPro Academy Z-Score</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>【節税と確定申告】米国株投資はどう申告するか？海外所得 750 萬 の免税枠と 30% 配当源泉徴収の実務</t>
+          <t>量的研究ワークフロー： 5MA、ボラティリティ、バックテストを同じ証拠チェーンに組み込む。</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -5879,7 +5879,7 @@
         </is>
       </c>
       <c r="J106" s="2" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -5896,12 +5896,12 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/09-high-dividend-etf-trap.html</t>
+          <t>ja/articles/investment/16-futures-pairs-basis.html</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/09-high-dividend-etf-trap.html</t>
+          <t>https://gugopro.com/ja/articles/investment/16-futures-pairs-basis.html</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -5911,12 +5911,12 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>【高配当 ETF 評価】台湾上場 ETF 00878/00919/00929 vs 米国 ETF SCHD：高配当利回りの罠を解くと総リターンの真実が見える | GugoPro Academy</t>
+          <t>臺指期／富台期のペア取引と期現價差：Basisからロールリスクまで｜GugoPro Academy</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>【高配当 ETF 評価】台湾上場 ETF 00878/00919/00929 vs 米国 ETF SCHD：高配当利回りの罠を解くと総リターンの真実が見える</t>
+          <t>臺指期／富台期ペア取引： まず Basis を分解し、その後で裁定について議論する。</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
@@ -5930,7 +5930,7 @@
         </is>
       </c>
       <c r="J107" s="2" t="n">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -5947,12 +5947,12 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/10-bond-investing-guide.html</t>
+          <t>ja/articles/investment/17-practical-trading.html</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/10-bond-investing-guide.html</t>
+          <t>https://gugopro.com/ja/articles/investment/17-practical-trading.html</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5962,12 +5962,12 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>【債券投資ガイド】米国債 (TLT/IEF) vs 投資適格社債 (LQD)：利下げサイクルにおける資産配分戦略 | GugoPro Academy</t>
+          <t>第13類 実戦取引：取引計画、実行、リスク管理、レビューの完全なナレッジツリー｜GugoPro Academy</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>【債券投資ガイド】米国債 (TLT/IEF) vs 投資適格社債 (LQD)：利下げサイクルにおける資産配分戦略</t>
+          <t>実戦トレーディング： アイデアを実行可能でストップが設定でき、再検討できるプロセスにする。</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -5981,7 +5981,7 @@
         </is>
       </c>
       <c r="J108" s="2" t="n">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -5998,12 +5998,12 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/11-brokerage-deep-review.html</t>
+          <t>ja/articles/investment/18-trend-following-breakout-playbook.html</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/11-brokerage-deep-review.html</t>
+          <t>https://gugopro.com/ja/articles/investment/18-trend-following-breakout-playbook.html</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
@@ -6013,12 +6013,12 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>【海外証券会社評価大全】IB（盈透／Interactive Brokers）、Firstrade、Charles Schwab（嘉信理財）─ 長所・短所、安全性と隠れたコスト比較 | GugoPro Academy</t>
+          <t>トレンド追跡とブレイクアウト戦略プレイブック：ルール、ポジション、フェイクブレイク、バックテスト検証｜GugoPro Academy</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>【海外証券会社評価大全】IB（盈透／Interactive Brokers）、Firstrade、Charles Schwab（嘉信理財）─ 長所・短所、安全性と隠れたコスト比較</t>
+          <t>トレンド追跡とブレイクアウト戦略： 自分の「見解」を検証可能なルールに書き換える。</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -6032,7 +6032,7 @@
         </is>
       </c>
       <c r="J109" s="2" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6044,17 +6044,17 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/12-inflation-hedging-reits-gold.html</t>
+          <t>ja/articles/investment/index.html</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/12-inflation-hedging-reits-gold.html</t>
+          <t>https://gugopro.com/ja/articles/investment/index.html</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -6064,12 +6064,12 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>【ヘッジ資産】金（GLD）と不動産投資信託（REITs）はインフレ対策として資産配分にどう組み込むか？ | GugoPro Academy</t>
+          <t>投資教育アカデミー | GugoPro Academy</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>【ヘッジ資産】金（GLD）と不動産投資信託（REITs）はインフレ対策として資産配分にどう組み込むか？</t>
+          <t>システム化 投資教育と実戦のマトリクス</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -6083,7 +6083,7 @@
         </is>
       </c>
       <c r="J110" s="2" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6100,12 +6100,12 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/13-technical-indicators-truth.html</t>
+          <t>ja/articles/modern-ziwei-guide.html</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/13-technical-indicators-truth.html</t>
+          <t>https://gugopro.com/ja/articles/modern-ziwei-guide.html</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -6115,12 +6115,12 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>【テクニカル分析の真実】移動平均線 (MA)、RSI、MACD は本当に役立つのか？クオンツトレーダーが見るテクニカル指標の有効場面と盲点 | GugoPro Academy</t>
+          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>【テクニカル分析の真実】移動平均線 (MA)、RSI、MACD は本当に役立つのか？クオンツトレーダーが見るテクニカル指標の有効場面と盲点</t>
+          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -6134,10 +6134,10 @@
         </is>
       </c>
       <c r="J111" s="2" t="n">
-        <v>80</v>
+        <v>169</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112">
@@ -6151,12 +6151,12 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/14-backtesting-overfitting-guide.html</t>
+          <t>ja/articles/shadowing-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/14-backtesting-overfitting-guide.html</t>
+          <t>https://gugopro.com/ja/articles/shadowing-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -6166,12 +6166,12 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>【システムトレード】バックテスト (Backtesting/回測) とは？過学習 (Overfitting/過度擬合) と歴史的罠を避ける方法 | GugoPro Academy</t>
+          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈出力、AIチューターによるスピーキング実践ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>【システムトレード】バックテスト (Backtesting/回測) とは？過学習 (Overfitting/過度擬合) と歴史的罠を避ける方法</t>
+          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈輸出、AIチューターによるスピーキング実践ガイド</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -6185,10 +6185,10 @@
         </is>
       </c>
       <c r="J112" s="2" t="n">
-        <v>95</v>
+        <v>146</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113">
@@ -6202,12 +6202,12 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/15-quant-research-workflow.html</t>
+          <t>ja/articles/tarot-decision-framework.html</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/15-quant-research-workflow.html</t>
+          <t>https://gugopro.com/ja/articles/tarot-decision-framework.html</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -6217,12 +6217,12 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>量的研究ワークフロー：5MAオフセット、ボラティリティのZ‑Score、アウト‑オブ‑サンプルバックテスト｜GugoPro Academy Z-Score</t>
+          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>量的研究ワークフロー： 5MA、ボラティリティ、バックテストを同じ証拠チェーンに組み込む。</t>
+          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
@@ -6236,10 +6236,10 @@
         </is>
       </c>
       <c r="J113" s="2" t="n">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114">
@@ -6253,12 +6253,12 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/16-futures-pairs-basis.html</t>
+          <t>ja/articles/tblt-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/16-futures-pairs-basis.html</t>
+          <t>https://gugopro.com/ja/articles/tblt-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -6268,12 +6268,12 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>臺指期／富台期のペア取引と期現價差：Basisからロールリスクまで｜GugoPro Academy</t>
+          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>臺指期／富台期ペア取引： まず Basis を分解し、その後で裁定について議論する。</t>
+          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
@@ -6287,10 +6287,10 @@
         </is>
       </c>
       <c r="J114" s="2" t="n">
-        <v>84</v>
+        <v>184</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115">
@@ -6304,12 +6304,12 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/17-practical-trading.html</t>
+          <t>ja/articles/tdee-and-macros-guide.html</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/17-practical-trading.html</t>
+          <t>https://gugopro.com/ja/articles/tdee-and-macros-guide.html</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -6319,12 +6319,12 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>第13類 実戦取引：取引計画、実行、リスク管理、レビューの完全なナレッジツリー｜GugoPro Academy</t>
+          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル｜GugoPro 代謝健康專欄</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>実戦トレーディング： アイデアを実行可能でストップが設定でき、再検討できるプロセスにする。</t>
+          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -6338,10 +6338,10 @@
         </is>
       </c>
       <c r="J115" s="2" t="n">
-        <v>89</v>
+        <v>248</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="116">
@@ -6355,12 +6355,12 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/18-trend-following-breakout-playbook.html</t>
+          <t>ja/articles/travel-translator-guide.html</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/18-trend-following-breakout-playbook.html</t>
+          <t>https://gugopro.com/ja/articles/travel-translator-guide.html</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -6370,12 +6370,12 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>トレンド追跡とブレイクアウト戦略プレイブック：ルール、ポジション、フェイクブレイク、バックテスト検証｜GugoPro Academy</t>
+          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド｜GugoPro 異文化コミュニケーションコラム</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>トレンド追跡とブレイクアウト戦略： 自分の「見解」を検証可能なルールに書き換える。</t>
+          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
@@ -6389,10 +6389,10 @@
         </is>
       </c>
       <c r="J116" s="2" t="n">
-        <v>117</v>
+        <v>206</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117">
@@ -6401,17 +6401,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/investment/index.html</t>
+          <t>ja/articles/weight-loss-planner-guide.html</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/investment/index.html</t>
+          <t>https://gugopro.com/ja/articles/weight-loss-planner-guide.html</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -6421,12 +6421,12 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>投資教育アカデミー | GugoPro Academy</t>
+          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド｜GugoPro 運動生理学コラム</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>システム化 投資教育と実戦のマトリクス</t>
+          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
@@ -6440,10 +6440,10 @@
         </is>
       </c>
       <c r="J117" s="2" t="n">
-        <v>68</v>
+        <v>229</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118">
@@ -6457,12 +6457,12 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/modern-ziwei-guide.html</t>
+          <t>ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/modern-ziwei-guide.html</t>
+          <t>https://gugopro.com/ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -6472,12 +6472,12 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ｜GugoPro 意思決定科学コラム</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイングで母語レベルの聴覚神経回路を構築する完全ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
@@ -6491,7 +6491,7 @@
         </is>
       </c>
       <c r="J118" s="2" t="n">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>2</v>
@@ -6508,12 +6508,12 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/shadowing-with-ai-tutor.html</t>
+          <t>ja/articles/youtube-listening-connected-speech-guide.html</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/shadowing-with-ai-tutor.html</t>
+          <t>https://gugopro.com/ja/articles/youtube-listening-connected-speech-guide.html</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -6523,12 +6523,12 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈出力、AIチューターによるスピーキング実践ガイド｜GugoPro 言語科学コラム</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイング完全ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈輸出、AIチューターによるスピーキング実践ガイド</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
@@ -6542,7 +6542,7 @@
         </is>
       </c>
       <c r="J119" s="2" t="n">
-        <v>146</v>
+        <v>170</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>2</v>
@@ -6559,12 +6559,12 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/tarot-decision-framework.html</t>
+          <t>ja/articles/youtube-sequel-tracker-guide.html</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/tarot-decision-framework.html</t>
+          <t>https://gugopro.com/ja/articles/youtube-sequel-tracker-guide.html</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -6574,12 +6574,12 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル｜GugoPro 意思決定科学コラム</t>
+          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消しNLP正規表現ノイズ除去と差分照合で跨チャンネル追跡を実現する｜GugoPro ストリーミング研究コラム</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル</t>
+          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消し NLP正規表現ノイズ除去と差分照合 で跨チャンネル追跡を実現する</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
@@ -6593,7 +6593,7 @@
         </is>
       </c>
       <c r="J120" s="2" t="n">
-        <v>161</v>
+        <v>224</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>2</v>
@@ -6605,17 +6605,17 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/tblt-with-ai-tutor.html</t>
+          <t>ja/tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/tblt-with-ai-tutor.html</t>
+          <t>https://gugopro.com/ja/tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -6625,12 +6625,12 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド｜GugoPro 言語科学コラム</t>
+          <t>リダイレクト中 - AI多言語スピーキングチューター | GugoPro</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
@@ -6640,14 +6640,14 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J121" s="2" t="n">
-        <v>184</v>
+        <v>0</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -6656,17 +6656,17 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/tdee-and-macros-guide.html</t>
+          <t>ja/tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/tdee-and-macros-guide.html</t>
+          <t>https://gugopro.com/ja/tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -6676,12 +6676,12 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル｜GugoPro 代謝健康專欄</t>
+          <t>リダイレクト中 - 対面型リアルタイム音声翻訳 | GugoPro</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
@@ -6691,14 +6691,14 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J122" s="2" t="n">
-        <v>248</v>
+        <v>0</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -6707,17 +6707,17 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/travel-translator-guide.html</t>
+          <t>ja/tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/travel-translator-guide.html</t>
+          <t>https://gugopro.com/ja/tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -6727,12 +6727,12 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド｜GugoPro 異文化コミュニケーションコラム</t>
+          <t>リダイレクト中 - AIタロットマスター | GugoPro</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
@@ -6742,14 +6742,14 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J123" s="2" t="n">
-        <v>206</v>
+        <v>0</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124">
@@ -6758,17 +6758,17 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/weight-loss-planner-guide.html</t>
+          <t>ja/tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/weight-loss-planner-guide.html</t>
+          <t>https://gugopro.com/ja/tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -6778,12 +6778,12 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド｜GugoPro 運動生理学コラム</t>
+          <t>リダイレクト中 - AI紫微斗数マスター | GugoPro</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
@@ -6793,14 +6793,14 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J124" s="2" t="n">
-        <v>229</v>
+        <v>0</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125">
@@ -6809,17 +6809,17 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
+          <t>ja/tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
+          <t>https://gugopro.com/ja/tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
@@ -6829,12 +6829,12 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイングで母語レベルの聴覚神経回路を構築する完全ガイド｜GugoPro 言語科学コラム</t>
+          <t>リダイレクト中 - YouTube続編追跡 | GugoPro</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -6844,14 +6844,14 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J125" s="2" t="n">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126">
@@ -6860,17 +6860,17 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/youtube-listening-connected-speech-guide.html</t>
+          <t>ja/tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/youtube-listening-connected-speech-guide.html</t>
+          <t>https://gugopro.com/ja/tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -6880,12 +6880,12 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイング完全ガイド｜GugoPro 言語科学コラム</t>
+          <t>リダイレクト中 - YouTube学習プレイヤー | GugoPro</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -6895,14 +6895,14 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J126" s="2" t="n">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -6911,17 +6911,17 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/youtube-sequel-tracker-guide.html</t>
+          <t>ja/tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/youtube-sequel-tracker-guide.html</t>
+          <t>https://gugopro.com/ja/tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -6931,12 +6931,12 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消しNLP正規表現ノイズ除去と差分照合で跨チャンネル追跡を実現する｜GugoPro ストリーミング研究コラム</t>
+          <t>リダイレクト中 - AI栄養士 | GugoPro</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消し NLP正規表現ノイズ除去と差分照合 で跨チャンネル追跡を実現する</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -6946,14 +6946,14 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J127" s="2" t="n">
-        <v>224</v>
+        <v>0</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -6962,17 +6962,17 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>ja/legal/about.html</t>
+          <t>ja/tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/legal/about.html</t>
+          <t>https://gugopro.com/ja/tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -6982,12 +6982,12 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>GugoProについて | GugoPro</t>
+          <t>リダイレクト中 - AI減量コーチ | GugoPro</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>GugoProについて</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
@@ -6997,14 +6997,14 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J128" s="2" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="K128" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -7018,27 +7018,27 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>ja/legal/contact.html</t>
+          <t>privacy.html</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/legal/contact.html</t>
+          <t>https://gugopro.com/privacy.html</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>お問い合わせ | GugoPro</t>
+          <t>隱私權政策｜GugoPro</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>お問い合わせ</t>
+          <t>隱私權政策</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
@@ -7052,7 +7052,7 @@
         </is>
       </c>
       <c r="J129" s="2" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="K129" s="2" t="n">
         <v>0</v>
@@ -7069,27 +7069,27 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>ja/legal/disclaimer.html</t>
+          <t>terms.html</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/legal/disclaimer.html</t>
+          <t>https://gugopro.com/terms.html</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>免責事項 | GugoPro</t>
+          <t>服務條款｜GugoPro</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>免責事項</t>
+          <t>服務條款</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -7103,7 +7103,7 @@
         </is>
       </c>
       <c r="J130" s="2" t="n">
-        <v>142</v>
+        <v>49</v>
       </c>
       <c r="K130" s="2" t="n">
         <v>0</v>
@@ -7115,32 +7115,32 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>ja/legal/privacy.html</t>
+          <t>tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/legal/privacy.html</t>
+          <t>https://gugopro.com/tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>プライバシーポリシー | GugoPro</t>
+          <t>AI多國語言對話導師</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>プライバシーポリシー</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -7154,10 +7154,10 @@
         </is>
       </c>
       <c r="J131" s="2" t="n">
-        <v>136</v>
+        <v>65</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -7166,32 +7166,32 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>ja/legal/terms.html</t>
+          <t>tools/ai/gemini-api-quota.html</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/legal/terms.html</t>
+          <t>https://gugopro.com/tools/ai/gemini-api-quota.html</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>利用規約 | GugoPro</t>
+          <t>Gemini API 配額服務導覽｜GugoPro</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>利用規約</t>
+          <t>Gemini API 配額服務導覽</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -7205,7 +7205,7 @@
         </is>
       </c>
       <c r="J132" s="2" t="n">
-        <v>129</v>
+        <v>61</v>
       </c>
       <c r="K132" s="2" t="n">
         <v>0</v>
@@ -7217,27 +7217,27 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/english-speaking-tutor.html</t>
+          <t>tools/ai/nutritionist.html</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/english-speaking-tutor.html</t>
+          <t>https://gugopro.com/tools/ai/nutritionist.html</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AI多言語スピーキングチューター | GugoPro</t>
+          <t>AI 專屬營養師｜AI 營養諮詢、TDEE 與飲食紀錄工具、免安裝與隱私說明 - GugoPro</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -7252,11 +7252,11 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J133" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K133" s="2" t="n">
         <v>1</v>
@@ -7273,27 +7273,27 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/realtime-translator.html</t>
+          <t>tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/realtime-translator.html</t>
+          <t>https://gugopro.com/tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - 対面型リアルタイム音声翻訳 | GugoPro</t>
+          <t>面對面旅遊對話翻譯｜出國旅遊即時翻譯與雙向語音對話｜GugoPro</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>面對面旅遊對話翻譯：出國旅遊即時翻譯與雙向語音對話</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
@@ -7303,14 +7303,14 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J134" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="K134" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="K134" s="2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -7324,22 +7324,22 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/tarot-master.html</t>
+          <t>tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/tarot-master.html</t>
+          <t>https://gugopro.com/tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AIタロットマスター | GugoPro</t>
+          <t>AI 塔羅大師｜五種塔羅牌陣、提問指南與自我反思 - GugoPro</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -7354,11 +7354,11 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J135" s="2" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="K135" s="2" t="n">
         <v>1</v>
@@ -7375,27 +7375,27 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/ziwei-astrology.html</t>
+          <t>tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/ziwei-astrology.html</t>
+          <t>https://gugopro.com/tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AI紫微斗数マスター | GugoPro</t>
+          <t>AI 紫微斗數大師｜紫微斗數線上排盤資料整理與十二宮位指南 - GugoPro</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>把命盤問題，整理成可行動的洞察</t>
         </is>
       </c>
       <c r="H136" s="2" t="inlineStr">
@@ -7405,11 +7405,11 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J136" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="K136" s="2" t="n">
         <v>1</v>
@@ -7426,44 +7426,44 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai-media/ai-video-tracker.html</t>
+          <t>tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai-media/ai-video-tracker.html</t>
+          <t>https://gugopro.com/tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - YouTube続編追跡 | GugoPro</t>
+          <t>YouTube 續集與新季追蹤器 - GugoPro</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
+          <t>YouTube 續集與新季追蹤器</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>可見</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
           <t>❌ 缺失</t>
         </is>
       </c>
-      <c r="H137" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I137" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
       <c r="J137" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="K137" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="K137" s="2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="138">
@@ -7472,32 +7472,32 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/english/l-player-study.html</t>
+          <t>tools/compound-interest.html</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/english/l-player-study.html</t>
+          <t>https://gugopro.com/tools/compound-interest.html</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - YouTube学習プレイヤー | GugoPro</t>
+          <t>Compound Interest 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>進階複利與退休目標規劃計算機</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -7507,14 +7507,14 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J138" s="2" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139">
@@ -7528,41 +7528,41 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/health/tdee-macros-calculator.html</t>
+          <t>tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/health/tdee-macros-calculator.html</t>
+          <t>https://gugopro.com/tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AI栄養士 | GugoPro</t>
+          <t>【AB English Podcast】Ep.1 自我介紹與日常社交對話 (Mia &amp; Alex)｜L-Player</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>YouTube 影音「聽・寫・口說」多國語言跟讀器</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>可見</t>
+          <t>疑似隱藏</t>
         </is>
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J139" s="2" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="K139" s="2" t="n">
         <v>1</v>
@@ -7574,32 +7574,32 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/health/weight-loss-planner.html</t>
+          <t>tools/etf-dividend-calculator.html</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/health/weight-loss-planner.html</t>
+          <t>https://gugopro.com/tools/etf-dividend-calculator.html</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AI減量コーチ | GugoPro</t>
+          <t>Etf Dividend Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>把配息拆成一條， 看得懂的現金流曲線。</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -7609,14 +7609,14 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J140" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="K140" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="K140" s="2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="141">
@@ -7625,17 +7625,17 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>privacy.html</t>
+          <t>tools/finance/kelly-criterion-calculator.html</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/privacy.html</t>
+          <t>https://gugopro.com/tools/finance/kelly-criterion-calculator.html</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
@@ -7645,12 +7645,12 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>隱私權政策｜GugoPro</t>
+          <t>Kelly Criterion Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>隱私權政策</t>
+          <t>凱利公式與資金控管模擬器</t>
         </is>
       </c>
       <c r="H141" s="2" t="inlineStr">
@@ -7664,10 +7664,10 @@
         </is>
       </c>
       <c r="J141" s="2" t="n">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K141" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -7676,17 +7676,17 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>quant/pine-script-basics.html</t>
+          <t>tools/finance/sports-hedging-calculator.html</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/quant/pine-script-basics.html</t>
+          <t>https://gugopro.com/tools/finance/sports-hedging-calculator.html</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -7696,12 +7696,12 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>Unit 4.2: TradingView Pine Script 程式交易入門 | GugoPro 財經教學學院</t>
+          <t>Sports Hedging Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>TradingView Pine Script 程式交易入門與指標開發</t>
+          <t>運動彩券賠率換算與套利對沖計算器</t>
         </is>
       </c>
       <c r="H142" s="2" t="inlineStr">
@@ -7715,10 +7715,10 @@
         </is>
       </c>
       <c r="J142" s="2" t="n">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="K142" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -7727,32 +7727,32 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>support.html</t>
+          <t>tools/games/mahjong-waits-calculator.html</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/support.html</t>
+          <t>https://gugopro.com/tools/games/mahjong-waits-calculator.html</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>zh-TW</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>GugoPro｜贊助支持</t>
+          <t>Mahjong Waits Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>支持 GugoPro</t>
+          <t>麻將聽牌張數與進張勝率計算器</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
@@ -7766,7 +7766,7 @@
         </is>
       </c>
       <c r="J143" s="2" t="n">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="K143" s="2" t="n">
         <v>0</v>
@@ -7778,17 +7778,17 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>法律條款</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>terms.html</t>
+          <t>tools/games/poker-odds-calculator.html</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/terms.html</t>
+          <t>https://gugopro.com/tools/games/poker-odds-calculator.html</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -7798,12 +7798,12 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>服務條款｜GugoPro</t>
+          <t>Poker Odds Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>服務條款</t>
+          <t>德州撲克即時勝率計算器 Texas Hold'em Odds Calculator</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr">
@@ -7817,7 +7817,7 @@
         </is>
       </c>
       <c r="J144" s="2" t="n">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="K144" s="2" t="n">
         <v>0</v>
@@ -7829,32 +7829,32 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/english-speaking-tutor.html</t>
+          <t>tools/gaming/gacha-odds-calculator.html</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/english-speaking-tutor.html</t>
+          <t>https://gugopro.com/tools/gaming/gacha-odds-calculator.html</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>zh-TW</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>AI多國語言對話導師</t>
+          <t>Gacha Odds Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>Gacha Odds &amp; Pity Simulator v5</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
@@ -7868,10 +7868,10 @@
         </is>
       </c>
       <c r="J145" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -7885,12 +7885,12 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/gemini-api-quota.html</t>
+          <t>tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/gemini-api-quota.html</t>
+          <t>https://gugopro.com/tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
@@ -7900,12 +7900,12 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Gemini API 配額服務導覽｜GugoPro</t>
+          <t>AI 專屬營養師 | GugoPro</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>Gemini API 配額服務導覽</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
@@ -7919,10 +7919,10 @@
         </is>
       </c>
       <c r="J146" s="2" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K146" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -7931,17 +7931,17 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>歷史工具</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/nutritionist.html</t>
+          <t>tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/nutritionist.html</t>
+          <t>https://gugopro.com/tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>AI 專屬營養師｜AI 營養諮詢、TDEE 與飲食紀錄工具、免安裝與隱私說明 - GugoPro</t>
+          <t>AI減肥瘦身教練｜科學減脂與熱量赤字規劃 | GugoPro</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -7970,7 +7970,7 @@
         </is>
       </c>
       <c r="J147" s="2" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K147" s="2" t="n">
         <v>1</v>
@@ -7982,17 +7982,17 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/realtime-translator.html</t>
+          <t>tools/pdf/pdf-suite.html</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/realtime-translator.html</t>
+          <t>https://gugopro.com/tools/pdf/pdf-suite.html</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -8002,12 +8002,12 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>面對面旅遊對話翻譯｜出國旅遊即時翻譯與雙向語音對話｜GugoPro</t>
+          <t>PDF 全能工作站｜免安裝線上閱讀、合併、分割與標註、零檔案外洩 - GugoPro</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>面對面旅遊對話翻譯：出國旅遊即時翻譯與雙向語音對話</t>
+          <t>先選擇要處理的文件</t>
         </is>
       </c>
       <c r="H148" s="2" t="inlineStr">
@@ -8017,14 +8017,14 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J148" s="2" t="n">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="K148" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -8033,17 +8033,17 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/tarot-master.html</t>
+          <t>tools/poker/poker-odds-calculator.html</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/tarot-master.html</t>
+          <t>https://gugopro.com/tools/poker/poker-odds-calculator.html</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
@@ -8053,12 +8053,12 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>AI 塔羅大師｜五種塔羅牌陣、提問指南與自我反思 - GugoPro</t>
+          <t>Poker Odds Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>德州撲克即時勝率計算器 Texas Hold'em Odds Calculator</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
@@ -8072,10 +8072,10 @@
         </is>
       </c>
       <c r="J149" s="2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K149" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -8084,32 +8084,32 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/ziwei-astrology.html</t>
+          <t>tools/realestate-amortization.html</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/ziwei-astrology.html</t>
+          <t>https://gugopro.com/tools/realestate-amortization.html</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>zh-TW</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>AI 紫微斗數大師｜紫微斗數線上排盤資料整理與十二宮位指南 - GugoPro</t>
+          <t>Realestate Amortization 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>把命盤問題，整理成可行動的洞察</t>
+          <t>房貸本息攤還、利息與提前還款工具</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
@@ -8123,10 +8123,10 @@
         </is>
       </c>
       <c r="J150" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K150" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -8135,32 +8135,32 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>tools/ai-media/ai-video-tracker.html</t>
+          <t>tools/risk-reward-calculator.html</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai-media/ai-video-tracker.html</t>
+          <t>https://gugopro.com/tools/risk-reward-calculator.html</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>zh-TW</t>
+          <t>zh-Hant</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>YouTube 續集與新季追蹤器 - GugoPro</t>
+          <t>Risk Reward Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>YouTube 續集與新季追蹤器</t>
+          <t>先看即時價格，再決定風險。</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -8170,11 +8170,11 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J151" s="2" t="n">
-        <v>112</v>
+        <v>67</v>
       </c>
       <c r="K151" s="2" t="n">
         <v>0</v>
@@ -8191,12 +8191,12 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>tools/compound-interest.html</t>
+          <t>tools/tradingview-guide.html</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/compound-interest.html</t>
+          <t>https://gugopro.com/tools/tradingview-guide.html</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
@@ -8206,12 +8206,12 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>Compound Interest 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
+          <t>Tradingview Guide 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>進階複利與退休目標規劃計算機</t>
+          <t>全球最強圖表工具 TradingView</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
@@ -8228,7 +8228,7 @@
         <v>62</v>
       </c>
       <c r="K152" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="153">
@@ -8237,17 +8237,17 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>tools/english/l-player-study.html</t>
+          <t>tools/tutorials/how-to-get-gemini-api-key.html</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/english/l-player-study.html</t>
+          <t>https://gugopro.com/tools/tutorials/how-to-get-gemini-api-key.html</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
@@ -8257,17 +8257,17 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>【AB English Podcast】Ep.1 自我介紹與日常社交對話 (Mia &amp; Alex)｜L-Player</t>
+          <t>Gemini API Key 申請教學｜Google Gemini API Key 取得與安全設定教學、免安裝與隱私說明 - GugoPro</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>YouTube 影音「聽・寫・口說」多國語言跟讀器</t>
+          <t>Google Gemini API Key 1 分鐘快速申請步驟</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>疑似隱藏</t>
+          <t>可見</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
@@ -8276,7 +8276,7 @@
         </is>
       </c>
       <c r="J153" s="2" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="K153" s="2" t="n">
         <v>1</v>
@@ -8293,27 +8293,27 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>tools/etf-dividend-calculator.html</t>
+          <t>tools/tw-market/taiwan-pair-trading.html</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/etf-dividend-calculator.html</t>
+          <t>https://gugopro.com/tools/tw-market/taiwan-pair-trading.html</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>zh-Hant</t>
+          <t>zh-Hant-TW</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>Etf Dividend Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
+          <t>Taiwan Pair Trading 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>把配息拆成一條， 看得懂的現金流曲線。</t>
+          <t>台灣股票與期貨 配對交易掃描工作站</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -8327,728 +8327,14 @@
         </is>
       </c>
       <c r="J154" s="2" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="K154" s="2" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="2" t="n">
-        <v>154</v>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C155" s="2" t="inlineStr">
-        <is>
-          <t>tools/finance/kelly-criterion-calculator.html</t>
-        </is>
-      </c>
-      <c r="D155" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/finance/kelly-criterion-calculator.html</t>
-        </is>
-      </c>
-      <c r="E155" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F155" s="2" t="inlineStr">
-        <is>
-          <t>Kelly Criterion Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G155" s="2" t="inlineStr">
-        <is>
-          <t>凱利公式與資金控管模擬器</t>
-        </is>
-      </c>
-      <c r="H155" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I155" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J155" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="K155" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="n">
-        <v>155</v>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C156" s="2" t="inlineStr">
-        <is>
-          <t>tools/finance/sports-hedging-calculator.html</t>
-        </is>
-      </c>
-      <c r="D156" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/finance/sports-hedging-calculator.html</t>
-        </is>
-      </c>
-      <c r="E156" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F156" s="2" t="inlineStr">
-        <is>
-          <t>Sports Hedging Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G156" s="2" t="inlineStr">
-        <is>
-          <t>運動彩券賠率換算與套利對沖計算器</t>
-        </is>
-      </c>
-      <c r="H156" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I156" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J156" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="K156" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="n">
-        <v>156</v>
-      </c>
-      <c r="B157" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C157" s="2" t="inlineStr">
-        <is>
-          <t>tools/games/mahjong-waits-calculator.html</t>
-        </is>
-      </c>
-      <c r="D157" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/games/mahjong-waits-calculator.html</t>
-        </is>
-      </c>
-      <c r="E157" s="2" t="inlineStr">
-        <is>
-          <t>zh-Hant</t>
-        </is>
-      </c>
-      <c r="F157" s="2" t="inlineStr">
-        <is>
-          <t>Mahjong Waits Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G157" s="2" t="inlineStr">
-        <is>
-          <t>麻將聽牌張數與進張勝率計算器</t>
-        </is>
-      </c>
-      <c r="H157" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I157" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J157" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="K157" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="n">
-        <v>157</v>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C158" s="2" t="inlineStr">
-        <is>
-          <t>tools/games/poker-odds-calculator.html</t>
-        </is>
-      </c>
-      <c r="D158" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/games/poker-odds-calculator.html</t>
-        </is>
-      </c>
-      <c r="E158" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F158" s="2" t="inlineStr">
-        <is>
-          <t>Poker Odds Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G158" s="2" t="inlineStr">
-        <is>
-          <t>德州撲克即時勝率計算器 Texas Hold'em Odds Calculator</t>
-        </is>
-      </c>
-      <c r="H158" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I158" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J158" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="K158" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="n">
-        <v>158</v>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C159" s="2" t="inlineStr">
-        <is>
-          <t>tools/gaming/gacha-odds-calculator.html</t>
-        </is>
-      </c>
-      <c r="D159" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/gaming/gacha-odds-calculator.html</t>
-        </is>
-      </c>
-      <c r="E159" s="2" t="inlineStr">
-        <is>
-          <t>zh-Hant</t>
-        </is>
-      </c>
-      <c r="F159" s="2" t="inlineStr">
-        <is>
-          <t>Gacha Odds Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G159" s="2" t="inlineStr">
-        <is>
-          <t>Gacha Odds &amp; Pity Simulator v5</t>
-        </is>
-      </c>
-      <c r="H159" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I159" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J159" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="K159" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="n">
-        <v>159</v>
-      </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C160" s="2" t="inlineStr">
-        <is>
-          <t>tools/health/tdee-macros-calculator.html</t>
-        </is>
-      </c>
-      <c r="D160" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/health/tdee-macros-calculator.html</t>
-        </is>
-      </c>
-      <c r="E160" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F160" s="2" t="inlineStr">
-        <is>
-          <t>AI 專屬營養師 | GugoPro</t>
-        </is>
-      </c>
-      <c r="G160" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H160" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I160" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J160" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="K160" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="n">
-        <v>160</v>
-      </c>
-      <c r="B161" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C161" s="2" t="inlineStr">
-        <is>
-          <t>tools/health/weight-loss-planner.html</t>
-        </is>
-      </c>
-      <c r="D161" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/health/weight-loss-planner.html</t>
-        </is>
-      </c>
-      <c r="E161" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F161" s="2" t="inlineStr">
-        <is>
-          <t>AI減肥瘦身教練｜科學減脂與熱量赤字規劃 | GugoPro</t>
-        </is>
-      </c>
-      <c r="G161" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H161" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I161" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J161" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="K161" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="2" t="n">
-        <v>161</v>
-      </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>tools/pdf/pdf-suite.html</t>
-        </is>
-      </c>
-      <c r="D162" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/pdf/pdf-suite.html</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>PDF 全能工作站｜免安裝線上閱讀、合併、分割與標註、零檔案外洩 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G162" s="2" t="inlineStr">
-        <is>
-          <t>先選擇要處理的文件</t>
-        </is>
-      </c>
-      <c r="H162" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I162" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="J162" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="K162" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="n">
-        <v>162</v>
-      </c>
-      <c r="B163" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t>tools/poker/poker-odds-calculator.html</t>
-        </is>
-      </c>
-      <c r="D163" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/poker/poker-odds-calculator.html</t>
-        </is>
-      </c>
-      <c r="E163" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F163" s="2" t="inlineStr">
-        <is>
-          <t>Poker Odds Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G163" s="2" t="inlineStr">
-        <is>
-          <t>德州撲克即時勝率計算器 Texas Hold'em Odds Calculator</t>
-        </is>
-      </c>
-      <c r="H163" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I163" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J163" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="K163" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="2" t="n">
-        <v>163</v>
-      </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t>tools/realestate-amortization.html</t>
-        </is>
-      </c>
-      <c r="D164" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/realestate-amortization.html</t>
-        </is>
-      </c>
-      <c r="E164" s="2" t="inlineStr">
-        <is>
-          <t>zh-Hant</t>
-        </is>
-      </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>Realestate Amortization 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G164" s="2" t="inlineStr">
-        <is>
-          <t>房貸本息攤還、利息與提前還款工具</t>
-        </is>
-      </c>
-      <c r="H164" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I164" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J164" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="K164" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="2" t="n">
-        <v>164</v>
-      </c>
-      <c r="B165" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t>tools/risk-reward-calculator.html</t>
-        </is>
-      </c>
-      <c r="D165" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/risk-reward-calculator.html</t>
-        </is>
-      </c>
-      <c r="E165" s="2" t="inlineStr">
-        <is>
-          <t>zh-Hant</t>
-        </is>
-      </c>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t>Risk Reward Calculator 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G165" s="2" t="inlineStr">
-        <is>
-          <t>先看即時價格，再決定風險。</t>
-        </is>
-      </c>
-      <c r="H165" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I165" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J165" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="K165" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="2" t="n">
-        <v>165</v>
-      </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>tools/tradingview-guide.html</t>
-        </is>
-      </c>
-      <c r="D166" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/tradingview-guide.html</t>
-        </is>
-      </c>
-      <c r="E166" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F166" s="2" t="inlineStr">
-        <is>
-          <t>Tradingview Guide 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G166" s="2" t="inlineStr">
-        <is>
-          <t>全球最強圖表工具 TradingView</t>
-        </is>
-      </c>
-      <c r="H166" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I166" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J166" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="K166" s="2" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="n">
-        <v>166</v>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>tools/tutorials/how-to-get-gemini-api-key.html</t>
-        </is>
-      </c>
-      <c r="D167" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/tutorials/how-to-get-gemini-api-key.html</t>
-        </is>
-      </c>
-      <c r="E167" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>Gemini API Key 申請教學｜Google Gemini API Key 取得與安全設定教學、免安裝與隱私說明 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G167" s="2" t="inlineStr">
-        <is>
-          <t>Google Gemini API Key 1 分鐘快速申請步驟</t>
-        </is>
-      </c>
-      <c r="H167" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I167" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J167" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="K167" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="n">
-        <v>167</v>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>tools/tw-market/taiwan-pair-trading.html</t>
-        </is>
-      </c>
-      <c r="D168" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/tw-market/taiwan-pair-trading.html</t>
-        </is>
-      </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t>zh-Hant-TW</t>
-        </is>
-      </c>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>Taiwan Pair Trading 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G168" s="2" t="inlineStr">
-        <is>
-          <t>台灣股票與期貨 配對交易掃描工作站</t>
-        </is>
-      </c>
-      <c r="H168" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I168" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J168" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="K168" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K168"/>
+  <autoFilter ref="A1:K154"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -9203,24 +8489,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId151"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId152"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId167"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId168"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId154"/>
   </tableParts>
 </worksheet>
 </file>
@@ -9257,7 +8529,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>167</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
@@ -9307,7 +8579,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -9317,7 +8589,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -9357,7 +8629,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Chore: remove locale tool redirect shells
</commit_message>
<xml_diff>
--- a/seo_inventory_report.xlsx
+++ b/seo_inventory_report.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SEO AdSense 盤點'!$A$1:$K$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SEO AdSense 盤點'!$A$1:$K$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -157,8 +157,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SEOInventory" displayName="SEOInventory" ref="A1:K96" headerRowCount="1">
-  <autoFilter ref="A1:K96"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SEOInventory" displayName="SEOInventory" ref="A1:K80" headerRowCount="1">
+  <autoFilter ref="A1:K80"/>
   <tableColumns count="11">
     <tableColumn id="1" name="編號"/>
     <tableColumn id="2" name="頁面分類"/>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K96"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2686,29 +2686,21 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/english-speaking-tutor.html</t>
+          <t>googled0dfad57039c64f6.html</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/english-speaking-tutor.html</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Redirecting - AI Multilingual Speaking Tutor | GugoPro</t>
-        </is>
-      </c>
+          <t>https://gugopro.com/googled0dfad57039c64f6.html</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
           <t>❌ 缺失</t>
@@ -2728,7 +2720,7 @@
         <v>0</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -2737,32 +2729,32 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/realtime-translator.html</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/realtime-translator.html</t>
+          <t>https://gugopro.com/index.html</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - Face-to-Face Travel Voice Translator | GugoPro</t>
+          <t>GugoPro 工具箱｜YouTube 雙語字幕學習、AI 翻譯塔羅、TDEE 減脂計算與 Gemini API 配額監控等 9 款免費工具</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>GugoPro 工具箱</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2772,14 +2764,14 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="46">
@@ -2788,17 +2780,17 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/tarot-master.html</t>
+          <t>index_en.html</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/tarot-master.html</t>
+          <t>https://gugopro.com/index_en.html</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2808,12 +2800,12 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - AI Tarot Master | GugoPro</t>
+          <t>GugoPro Hub | 9 Free Browser Tools for YouTube Study, AI Translation, Tarot, TDEE &amp; Gemini Quota</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>GugoPro Hub</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2823,14 +2815,14 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47">
@@ -2839,32 +2831,32 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>首頁</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai/ziwei-astrology.html</t>
+          <t>index_ja.html</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai/ziwei-astrology.html</t>
+          <t>https://gugopro.com/index_ja.html</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - GugoPro AI Ziwei Astrology Master | GugoPro</t>
+          <t>GugoPro ツールボックス｜YouTube 2言語字幕学習、AI 翻訳タロット、TDEE 減脂計算、Gemini API 配額監視など無料ブラウザツール9選</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>GugoPro ツールボックス</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2874,14 +2866,14 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48">
@@ -2890,32 +2882,32 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>en/tools/ai-media/ai-video-tracker.html</t>
+          <t>ja/articles/affective-filter-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/ai-media/ai-video-tracker.html</t>
+          <t>https://gugopro.com/ja/articles/affective-filter-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - YouTube Sequel Tracker | GugoPro</t>
+          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド｜GugoPro 言語学習コラム</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2925,14 +2917,14 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -2941,32 +2933,32 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>en/tools/english/l-player-study.html</t>
+          <t>ja/articles/amazon-ai-product-research-guide.html</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/english/l-player-study.html</t>
+          <t>https://gugopro.com/ja/articles/amazon-ai-product-research-guide.html</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - YouTube Study Player | GugoPro</t>
+          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス｜GugoPro EC戦略コラム</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2976,11 +2968,11 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>1</v>
@@ -2992,32 +2984,32 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>en/tools/health/tdee-macros-calculator.html</t>
+          <t>ja/articles/carb-cycling-and-home-workout-guide.html</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/health/tdee-macros-calculator.html</t>
+          <t>https://gugopro.com/ja/articles/carb-cycling-and-home-workout-guide.html</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - AI Nutritionist | GugoPro</t>
+          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意｜GugoPro 運動生理学コラム</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -3027,14 +3019,14 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -3043,32 +3035,32 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>en/tools/health/weight-loss-planner.html</t>
+          <t>ja/articles/diabetes-and-insulin-resistance-guide.html</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/en/tools/health/weight-loss-planner.html</t>
+          <t>https://gugopro.com/ja/articles/diabetes-and-insulin-resistance-guide.html</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Redirecting - AI Weight Loss Coach | GugoPro</t>
+          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控｜GugoPro 代謝医学コラム</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3078,14 +3070,14 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -3094,24 +3086,32 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>googled0dfad57039c64f6.html</t>
+          <t>ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/googled0dfad57039c64f6.html</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
+          <t>https://gugopro.com/ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル｜GugoPro 肝臓代謝コラム</t>
+        </is>
+      </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3121,14 +3121,14 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0</v>
+        <v>206</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -3137,32 +3137,32 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>index.html</t>
+          <t>ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/index.html</t>
+          <t>https://gugopro.com/ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>zh-TW</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>GugoPro 工具箱｜YouTube 雙語字幕學習、AI 翻譯塔羅、TDEE 減脂計算與 Gemini API 配額監控等 9 款免費工具</t>
+          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南｜GugoPro クラウドシステムコラム</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>GugoPro 工具箱</t>
+          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3176,10 +3176,10 @@
         </is>
       </c>
       <c r="J53" s="2" t="n">
-        <v>194</v>
+        <v>271</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -3188,32 +3188,32 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>index_en.html</t>
+          <t>ja/articles/how-to-master-tarot-guide.html</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/index_en.html</t>
+          <t>https://gugopro.com/ja/articles/how-to-master-tarot-guide.html</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>GugoPro Hub | 9 Free Browser Tools for YouTube Study, AI Translation, Tarot, TDEE &amp; Gemini Quota</t>
+          <t>タロットマスターへの道：78枚の丸暗記を脱し「直観的フロー・リーディング」へ——古典記号論、ナラティブ心理学、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>GugoPro Hub</t>
+          <t>如何にしてタロットマスターとなるか？ 78枚の意味の丸暗記から「直観的フロー・リーディング」へ：古典記号論・ナラティブ心理学・AI協同による限界的練習完全手引</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3227,10 +3227,10 @@
         </is>
       </c>
       <c r="J54" s="2" t="n">
-        <v>360</v>
+        <v>145</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -3239,17 +3239,17 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>首頁</t>
+          <t>專欄文章</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>index_ja.html</t>
+          <t>ja/articles/how-to-master-ziwei-guide.html</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/index_ja.html</t>
+          <t>https://gugopro.com/ja/articles/how-to-master-ziwei-guide.html</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3259,12 +3259,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>GugoPro ツールボックス｜YouTube 2言語字幕学習、AI 翻訳タロット、TDEE 減脂計算、Gemini API 配額監視など無料ブラウザツール9選</t>
+          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>GugoPro ツールボックス</t>
+          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3278,10 +3278,10 @@
         </is>
       </c>
       <c r="J55" s="2" t="n">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
@@ -3295,12 +3295,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/affective-filter-with-ai-tutor.html</t>
+          <t>ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/affective-filter-with-ai-tutor.html</t>
+          <t>https://gugopro.com/ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3310,12 +3310,12 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド｜GugoPro 言語学習コラム</t>
+          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド｜GugoPro 代謝内分泌コラム</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>話す恐怖を克服する心理学：クラッシェンの「情意フィルター仮説」、外国語不安（FLA）と AI チューターのゼロ圧力スピーキング完全ガイド</t>
+          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3329,7 +3329,7 @@
         </is>
       </c>
       <c r="J56" s="2" t="n">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>2</v>
@@ -3346,12 +3346,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/amazon-ai-product-research-guide.html</t>
+          <t>ja/articles/modern-ziwei-guide.html</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/amazon-ai-product-research-guide.html</t>
+          <t>https://gugopro.com/ja/articles/modern-ziwei-guide.html</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3361,12 +3361,12 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス｜GugoPro EC戦略コラム</t>
+          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>2026 越境EC・高精度リサーチ完全攻略：AIセマンティック・リバースエンジニアリングによるAmazonヒット商品開発、競合低評価（VOC）痛点分析とListingキーワード配置マトリクス</t>
+          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3380,10 +3380,10 @@
         </is>
       </c>
       <c r="J57" s="2" t="n">
-        <v>227</v>
+        <v>169</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
@@ -3397,12 +3397,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/carb-cycling-and-home-workout-guide.html</t>
+          <t>ja/articles/shadowing-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/carb-cycling-and-home-workout-guide.html</t>
+          <t>https://gugopro.com/ja/articles/shadowing-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3412,12 +3412,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意｜GugoPro 運動生理学コラム</t>
+          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈出力、AIチューターによるスピーキング実践ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>炭水化物循環法（カーボサイクル）完全減脂ガイド：高・低炭水化物日の生化学機序、器具不要の自宅燃焼ルーティン、筋分解防止の極意</t>
+          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈輸出、AIチューターによるスピーキング実践ガイド</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3431,7 +3431,7 @@
         </is>
       </c>
       <c r="J58" s="2" t="n">
-        <v>204</v>
+        <v>146</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>2</v>
@@ -3448,12 +3448,12 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/diabetes-and-insulin-resistance-guide.html</t>
+          <t>ja/articles/tarot-decision-framework.html</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/diabetes-and-insulin-resistance-guide.html</t>
+          <t>https://gugopro.com/ja/articles/tarot-decision-framework.html</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3463,12 +3463,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控｜GugoPro 代謝医学コラム</t>
+          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル｜GugoPro 意思決定科学コラム</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>糖尿病予備群・インスリン抵抗性の食事法完全ガイド：GI/GL値・カーボカウントからAI写真食事管理まで——血糖値スパイクを防ぐ栄養素調控</t>
+          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3482,7 +3482,7 @@
         </is>
       </c>
       <c r="J59" s="2" t="n">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>2</v>
@@ -3499,12 +3499,12 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
+          <t>ja/articles/tblt-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/fatty-liver-and-mediterranean-diet-guide.html</t>
+          <t>https://gugopro.com/ja/articles/tblt-with-ai-tutor.html</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3514,12 +3514,12 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル｜GugoPro 肝臓代謝コラム</t>
+          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>脂肪肝を逆転する減糖＆地中海食完全ガイド：内臓脂肪燃焼からPFC黄金比率・外食AI管理まで——MASLDを根本改善する長寿実戦マニュアル</t>
+          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3533,7 +3533,7 @@
         </is>
       </c>
       <c r="J60" s="2" t="n">
-        <v>206</v>
+        <v>184</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>2</v>
@@ -3550,12 +3550,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
+          <t>ja/articles/tdee-and-macros-guide.html</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/gemini-api-free-tier-and-developer-guide.html</t>
+          <t>https://gugopro.com/ja/articles/tdee-and-macros-guide.html</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3565,12 +3565,12 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南｜GugoPro クラウドシステムコラム</t>
+          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル｜GugoPro 代謝健康專欄</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>2026 開発者完全攻略ハンドブック：Google Gemini 公式無料APIを活用したゼロコスト商用グレードアプリのアーキテクチャ設計とエラー完全トラブルシューティング指南</t>
+          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3584,7 +3584,7 @@
         </is>
       </c>
       <c r="J61" s="2" t="n">
-        <v>271</v>
+        <v>248</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>2</v>
@@ -3601,12 +3601,12 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/how-to-master-tarot-guide.html</t>
+          <t>ja/articles/travel-translator-guide.html</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/how-to-master-tarot-guide.html</t>
+          <t>https://gugopro.com/ja/articles/travel-translator-guide.html</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3616,12 +3616,12 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>タロットマスターへの道：78枚の丸暗記を脱し「直観的フロー・リーディング」へ——古典記号論、ナラティブ心理学、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
+          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド｜GugoPro 異文化コミュニケーションコラム</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>如何にしてタロットマスターとなるか？ 78枚の意味の丸暗記から「直観的フロー・リーディング」へ：古典記号論・ナラティブ心理学・AI協同による限界的練習完全手引</t>
+          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3635,7 +3635,7 @@
         </is>
       </c>
       <c r="J62" s="2" t="n">
-        <v>145</v>
+        <v>206</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>2</v>
@@ -3652,12 +3652,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/how-to-master-ziwei-guide.html</t>
+          <t>ja/articles/weight-loss-planner-guide.html</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/how-to-master-ziwei-guide.html</t>
+          <t>https://gugopro.com/ja/articles/weight-loss-planner-guide.html</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -3667,12 +3667,12 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド｜GugoPro 意思決定科学コラム</t>
+          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド｜GugoPro 運動生理学コラム</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>紫微斗数マスターへの道：百の星の丸暗記を脱し「動態格局解盤」へ——文化記号論、システムダイナミクス、AI協同による限界的練習完全ガイド</t>
+          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3686,7 +3686,7 @@
         </is>
       </c>
       <c r="J63" s="2" t="n">
-        <v>199</v>
+        <v>229</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>2</v>
@@ -3703,12 +3703,12 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
+          <t>ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/intermittent-fasting-and-calorie-deficit-guide.html</t>
+          <t>https://gugopro.com/ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3718,12 +3718,12 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド｜GugoPro 代謝内分泌コラム</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイングで母語レベルの聴覚神経回路を構築する完全ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>168断食はカロリー計算より本当に痩せるのか？細胞自噬、インスリン仮説からエネルギー赤字の真相まで：リバウンドと筋肉減少の罠を解体する完全ガイド</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="J64" s="2" t="n">
-        <v>233</v>
+        <v>161</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>2</v>
@@ -3754,12 +3754,12 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/modern-ziwei-guide.html</t>
+          <t>ja/articles/youtube-listening-connected-speech-guide.html</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/modern-ziwei-guide.html</t>
+          <t>https://gugopro.com/ja/articles/youtube-listening-connected-speech-guide.html</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -3769,12 +3769,12 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ｜GugoPro 意思決定科学コラム</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイング完全ガイド｜GugoPro 言語科学コラム</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>宿命論とオカルト的脅迫からの脱却：現代心理学で再構築する紫微斗数——十二宮位、四化の動態からAI意思決定反省モデルへ</t>
+          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3788,7 +3788,7 @@
         </is>
       </c>
       <c r="J65" s="2" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>2</v>
@@ -3805,12 +3805,12 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/shadowing-with-ai-tutor.html</t>
+          <t>ja/articles/youtube-sequel-tracker-guide.html</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/shadowing-with-ai-tutor.html</t>
+          <t>https://gugopro.com/ja/articles/youtube-sequel-tracker-guide.html</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3820,12 +3820,12 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈出力、AIチューターによるスピーキング実践ガイド｜GugoPro 言語科学コラム</t>
+          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消しNLP正規表現ノイズ除去と差分照合で跨チャンネル追跡を実現する｜GugoPro ストリーミング研究コラム</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>「話せない英語」にサヨナラ！シャドーイング、CEFR文脈輸出、AIチューターによるスピーキング実践ガイド</t>
+          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消し NLP正規表現ノイズ除去と差分照合 で跨チャンネル追跡を実現する</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3839,7 +3839,7 @@
         </is>
       </c>
       <c r="J66" s="2" t="n">
-        <v>146</v>
+        <v>224</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>2</v>
@@ -3851,32 +3851,32 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>法律條款</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/tarot-decision-framework.html</t>
+          <t>privacy.html</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/tarot-decision-framework.html</t>
+          <t>https://gugopro.com/privacy.html</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル｜GugoPro 意思決定科学コラム</t>
+          <t>隱私權政策｜GugoPro</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>迷信的宿命論からの脱却：ユングの「元型」心理学・共時性からAIタロットへ——キャリアの二者択一と関係性不安を解体する構造化意思決定モデル</t>
+          <t>隱私權政策</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -3890,10 +3890,10 @@
         </is>
       </c>
       <c r="J67" s="2" t="n">
-        <v>161</v>
+        <v>60</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -3902,32 +3902,32 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>法律條款</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/tblt-with-ai-tutor.html</t>
+          <t>terms.html</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/tblt-with-ai-tutor.html</t>
+          <t>https://gugopro.com/terms.html</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド｜GugoPro 言語科学コラム</t>
+          <t>服務條款｜GugoPro</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>丸暗記にサヨナラ！タスク型教授法（TBLT）、Robinson認知仮説とAIチューターによる英会話実践ガイド</t>
+          <t>服務條款</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3941,10 +3941,10 @@
         </is>
       </c>
       <c r="J68" s="2" t="n">
-        <v>184</v>
+        <v>49</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -3953,32 +3953,32 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/tdee-and-macros-guide.html</t>
+          <t>tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/tdee-and-macros-guide.html</t>
+          <t>https://gugopro.com/tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル｜GugoPro 代謝健康專欄</t>
+          <t>AI多國語言對話導師</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>無駄な食事制限とリバウンドを完全に卒業！熱力学エネルギー収支、適応熱産生からAI食事解析まで：外食派のためのTDEE＆PFCバランス精密調整バイブル</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3992,10 +3992,10 @@
         </is>
       </c>
       <c r="J69" s="2" t="n">
-        <v>248</v>
+        <v>65</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -4004,32 +4004,32 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/travel-translator-guide.html</t>
+          <t>tools/ai/gemini-api-quota.html</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/travel-translator-guide.html</t>
+          <t>https://gugopro.com/tools/ai/gemini-api-quota.html</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド｜GugoPro 異文化コミュニケーションコラム</t>
+          <t>Gemini API 配額服務導覽｜GugoPro</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>スマホの気まずい手渡しにサヨナラ！180°対面反転UIのデザイン美学・HCI空間心理学と海外旅行会話実践ガイド</t>
+          <t>Gemini API 配額服務導覽</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -4043,10 +4043,10 @@
         </is>
       </c>
       <c r="J70" s="2" t="n">
-        <v>206</v>
+        <v>61</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -4055,32 +4055,32 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/weight-loss-planner-guide.html</t>
+          <t>tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/weight-loss-planner-guide.html</t>
+          <t>https://gugopro.com/tools/ai/realtime-translator.html</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド｜GugoPro 運動生理学コラム</t>
+          <t>面對面旅遊對話翻譯｜出國旅遊即時翻譯與雙向語音對話｜GugoPro</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>線形減量の幻想からの脱却！Wishnofsky 7700kcal法則の破綻からレジスタンストレーニング期分け・停滞期突破まで：動的減量計画とカロリー赤字完全ガイド</t>
+          <t>面對面旅遊對話翻譯：出國旅遊即時翻譯與雙向語音對話</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -4094,10 +4094,10 @@
         </is>
       </c>
       <c r="J71" s="2" t="n">
-        <v>229</v>
+        <v>82</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -4106,32 +4106,32 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
+          <t>tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/youtube-english-listening-and-shadowing-guide.html</t>
+          <t>https://gugopro.com/tools/ai/tarot-master.html</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイングで母語レベルの聴覚神経回路を構築する完全ガイド｜GugoPro 言語科学コラム</t>
+          <t>AI 塔羅大師｜五種塔羅牌陣、提問指南與自我反思 - GugoPro</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -4145,10 +4145,10 @@
         </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>161</v>
+        <v>63</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -4157,32 +4157,32 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/youtube-listening-connected-speech-guide.html</t>
+          <t>tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/youtube-listening-connected-speech-guide.html</t>
+          <t>https://gugopro.com/tools/ai/ziwei-astrology.html</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、レーベンシュタイン聴解、シャドーイング完全ガイド｜GugoPro 言語科学コラム</t>
+          <t>AI 紫微斗數大師｜紫微斗數線上排盤資料整理與十二宮位指南 - GugoPro</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>YouTube英語学習が挫折する真の理由とは？音韻知覚理論、 レーベンシュタイン聴解、シャドーイング で母語レベルの聴覚神経回路を構築する完全ガイド</t>
+          <t>把命盤問題，整理成可行動的洞察</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -4196,10 +4196,10 @@
         </is>
       </c>
       <c r="J73" s="2" t="n">
-        <v>170</v>
+        <v>70</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -4208,32 +4208,32 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>專欄文章</t>
+          <t>核心工具</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>ja/articles/youtube-sequel-tracker-guide.html</t>
+          <t>tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/articles/youtube-sequel-tracker-guide.html</t>
+          <t>https://gugopro.com/tools/ai-media/ai-video-tracker.html</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消しNLP正規表現ノイズ除去と差分照合で跨チャンネル追跡を実現する｜GugoPro ストリーミング研究コラム</t>
+          <t>YouTube 續集與新季追蹤器 - GugoPro</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2026年YouTube動画推薦アルゴリズムとシリーズ検索完全ガイド：推薦漏れを解消し NLP正規表現ノイズ除去と差分照合 で跨チャンネル追跡を実現する</t>
+          <t>YouTube 續集與新季追蹤器</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -4243,14 +4243,14 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>✅ 已配置</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="J74" s="2" t="n">
-        <v>224</v>
+        <v>112</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -4264,41 +4264,41 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/english-speaking-tutor.html</t>
+          <t>tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/english-speaking-tutor.html</t>
+          <t>https://gugopro.com/tools/english/l-player-study.html</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AI多言語スピーキングチューター | GugoPro</t>
+          <t>【AB English Podcast】Ep.1 自我介紹與日常社交對話 (Mia &amp; Alex)｜L-Player</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>YouTube 影音「聽・寫・口說」多國語言跟讀器</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>可見</t>
+          <t>疑似隱藏</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>1</v>
@@ -4315,22 +4315,22 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/realtime-translator.html</t>
+          <t>tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/realtime-translator.html</t>
+          <t>https://gugopro.com/tools/health/tdee-macros-calculator.html</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - 対面型リアルタイム音声翻訳 | GugoPro</t>
+          <t>AI 專屬營養師 | GugoPro</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4345,11 +4345,11 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>1</v>
@@ -4366,22 +4366,22 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/tarot-master.html</t>
+          <t>tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/tarot-master.html</t>
+          <t>https://gugopro.com/tools/health/weight-loss-planner.html</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AIタロットマスター | GugoPro</t>
+          <t>AI減肥瘦身教練｜科學減脂與熱量赤字規劃 | GugoPro</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -4396,11 +4396,11 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>1</v>
@@ -4412,32 +4412,32 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai/ziwei-astrology.html</t>
+          <t>tools/pdf/pdf-suite.html</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai/ziwei-astrology.html</t>
+          <t>https://gugopro.com/tools/pdf/pdf-suite.html</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - AI紫微斗数マスター | GugoPro</t>
+          <t>PDF 全能工作站｜免安裝線上閱讀、合併、分割與標註、零檔案外洩 - GugoPro</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>先選擇要處理的文件</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -4447,11 +4447,11 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>❌ 未配置（合規）</t>
         </is>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>1</v>
@@ -4463,32 +4463,32 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>實用教學</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/ai-media/ai-video-tracker.html</t>
+          <t>tools/tutorials/how-to-get-gemini-api-key.html</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/ai-media/ai-video-tracker.html</t>
+          <t>https://gugopro.com/tools/tutorials/how-to-get-gemini-api-key.html</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-TW</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - YouTube続編追跡 | GugoPro</t>
+          <t>Gemini API Key 申請教學｜Google Gemini API Key 取得與安全設定教學、免安裝與隱私說明 - GugoPro</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>Google Gemini API Key 1 分鐘快速申請步驟</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -4498,11 +4498,11 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>✅ 已配置</t>
         </is>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>1</v>
@@ -4514,32 +4514,32 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>核心工具</t>
+          <t>歷史工具</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>ja/tools/english/l-player-study.html</t>
+          <t>tools/tw-market/taiwan-pair-trading.html</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/ja/tools/english/l-player-study.html</t>
+          <t>https://gugopro.com/tools/tw-market/taiwan-pair-trading.html</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>zh-Hant-TW</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>リダイレクト中 - YouTube学習プレイヤー | GugoPro</t>
+          <t>Taiwan Pair Trading 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>台灣股票與期貨 配對交易掃描工作站</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4549,834 +4549,18 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>❌ 未配置（合規）</t>
         </is>
       </c>
       <c r="J80" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="K80" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="K80" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>ja/tools/health/tdee-macros-calculator.html</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/ja/tools/health/tdee-macros-calculator.html</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>リダイレクト中 - AI栄養士 | GugoPro</t>
-        </is>
-      </c>
-      <c r="G81" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="J81" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K81" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>ja/tools/health/weight-loss-planner.html</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/ja/tools/health/weight-loss-planner.html</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>リダイレクト中 - AI減量コーチ | GugoPro</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="J82" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K82" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>法律條款</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>privacy.html</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/privacy.html</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>隱私權政策｜GugoPro</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="inlineStr">
-        <is>
-          <t>隱私權政策</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I83" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J83" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="K83" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>法律條款</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>terms.html</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/terms.html</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>服務條款｜GugoPro</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>服務條款</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J84" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="K84" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>tools/ai/english-speaking-tutor.html</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/ai/english-speaking-tutor.html</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>AI多國語言對話導師</t>
-        </is>
-      </c>
-      <c r="G85" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I85" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J85" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="K85" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>tools/ai/gemini-api-quota.html</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/ai/gemini-api-quota.html</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>Gemini API 配額服務導覽｜GugoPro</t>
-        </is>
-      </c>
-      <c r="G86" s="2" t="inlineStr">
-        <is>
-          <t>Gemini API 配額服務導覽</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I86" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J86" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="K86" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>tools/ai/realtime-translator.html</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/ai/realtime-translator.html</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>面對面旅遊對話翻譯｜出國旅遊即時翻譯與雙向語音對話｜GugoPro</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="inlineStr">
-        <is>
-          <t>面對面旅遊對話翻譯：出國旅遊即時翻譯與雙向語音對話</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J87" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="K87" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>tools/ai/tarot-master.html</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/ai/tarot-master.html</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>AI 塔羅大師｜五種塔羅牌陣、提問指南與自我反思 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J88" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="K88" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>tools/ai/ziwei-astrology.html</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/ai/ziwei-astrology.html</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F89" s="2" t="inlineStr">
-        <is>
-          <t>AI 紫微斗數大師｜紫微斗數線上排盤資料整理與十二宮位指南 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G89" s="2" t="inlineStr">
-        <is>
-          <t>把命盤問題，整理成可行動的洞察</t>
-        </is>
-      </c>
-      <c r="H89" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I89" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J89" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="K89" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>tools/ai-media/ai-video-tracker.html</t>
-        </is>
-      </c>
-      <c r="D90" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/ai-media/ai-video-tracker.html</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>YouTube 續集與新季追蹤器 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G90" s="2" t="inlineStr">
-        <is>
-          <t>YouTube 續集與新季追蹤器</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I90" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="J90" s="2" t="n">
-        <v>112</v>
-      </c>
-      <c r="K90" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>tools/english/l-player-study.html</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/english/l-player-study.html</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>【AB English Podcast】Ep.1 自我介紹與日常社交對話 (Mia &amp; Alex)｜L-Player</t>
-        </is>
-      </c>
-      <c r="G91" s="2" t="inlineStr">
-        <is>
-          <t>YouTube 影音「聽・寫・口說」多國語言跟讀器</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="inlineStr">
-        <is>
-          <t>疑似隱藏</t>
-        </is>
-      </c>
-      <c r="I91" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J91" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="K91" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>tools/health/tdee-macros-calculator.html</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/health/tdee-macros-calculator.html</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>AI 專屬營養師 | GugoPro</t>
-        </is>
-      </c>
-      <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H92" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I92" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J92" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="K92" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>核心工具</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>tools/health/weight-loss-planner.html</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/health/weight-loss-planner.html</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr">
-        <is>
-          <t>AI減肥瘦身教練｜科學減脂與熱量赤字規劃 | GugoPro</t>
-        </is>
-      </c>
-      <c r="G93" s="2" t="inlineStr">
-        <is>
-          <t>❌ 缺失</t>
-        </is>
-      </c>
-      <c r="H93" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I93" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J93" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="K93" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="n">
-        <v>93</v>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>tools/pdf/pdf-suite.html</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/pdf/pdf-suite.html</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>PDF 全能工作站｜免安裝線上閱讀、合併、分割與標註、零檔案外洩 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>先選擇要處理的文件</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I94" s="2" t="inlineStr">
-        <is>
-          <t>❌ 未配置（合規）</t>
-        </is>
-      </c>
-      <c r="J94" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="K94" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="n">
-        <v>94</v>
-      </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>實用教學</t>
-        </is>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>tools/tutorials/how-to-get-gemini-api-key.html</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/tutorials/how-to-get-gemini-api-key.html</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>zh-TW</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>Gemini API Key 申請教學｜Google Gemini API Key 取得與安全設定教學、免安裝與隱私說明 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G95" s="2" t="inlineStr">
-        <is>
-          <t>Google Gemini API Key 1 分鐘快速申請步驟</t>
-        </is>
-      </c>
-      <c r="H95" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I95" s="2" t="inlineStr">
-        <is>
-          <t>✅ 已配置</t>
-        </is>
-      </c>
-      <c r="J95" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="K95" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>歷史工具</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>tools/tw-market/taiwan-pair-trading.html</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>https://gugopro.com/tools/tw-market/taiwan-pair-trading.html</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>zh-Hant-TW</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr">
-        <is>
-          <t>Taiwan Pair Trading 線上工具｜免安裝瀏覽器本機處理、零檔案外洩隱私 - GugoPro</t>
-        </is>
-      </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>台灣股票與期貨 配對交易掃描工作站</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr">
-        <is>
-          <t>可見</t>
-        </is>
-      </c>
-      <c r="I96" s="2" t="inlineStr">
-        <is>
-          <t>❌ 未配置（合規）</t>
-        </is>
-      </c>
-      <c r="J96" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="K96" s="2" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K96"/>
+  <autoFilter ref="A1:K80"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -5457,26 +4641,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId95"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId96"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId80"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5513,7 +4681,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
@@ -5533,7 +4701,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -5593,7 +4761,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -5603,7 +4771,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -5623,7 +4791,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>159</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: restore Amazon product research tool
</commit_message>
<xml_diff>
--- a/seo_inventory_report.xlsx
+++ b/seo_inventory_report.xlsx
@@ -2771,7 +2771,7 @@
         <v>194</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46">
@@ -3958,12 +3958,12 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/english-speaking-tutor.html</t>
+          <t>tools/ai/amazon-product-research.html</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/english-speaking-tutor.html</t>
+          <t>https://gugopro.com/tools/ai/amazon-product-research.html</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -3973,12 +3973,12 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>AI多國語言對話導師</t>
+          <t>Amazon AI 全品類智能選品導購 | GugoPro</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>❌ 缺失</t>
+          <t>🛒 Amazon AI 智能購物導師</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3992,7 +3992,7 @@
         </is>
       </c>
       <c r="J69" s="2" t="n">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>1</v>
@@ -4009,12 +4009,12 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>tools/ai/gemini-api-quota.html</t>
+          <t>tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>https://gugopro.com/tools/ai/gemini-api-quota.html</t>
+          <t>https://gugopro.com/tools/ai/english-speaking-tutor.html</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -4024,12 +4024,12 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Gemini API 配額服務導覽｜GugoPro</t>
+          <t>AI多國語言對話導師</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Gemini API 配額服務導覽</t>
+          <t>❌ 缺失</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -4043,10 +4043,10 @@
         </is>
       </c>
       <c r="J70" s="2" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>